<commit_message>
Consolidate blocks per David's Model: 5 variants -> 3 blocks
- Merge columns-media + columns-compare -> columns (base + compare variant)
- Merge cards-feature -> cards (base + feature variant)
- Update parsers (columns.js, cards.js), page-templates.json, import script
- Fix: cards parser no longer seeds a stray variant-name content row
- Re-imported content/cit.plain.html; all blocks render + variants styled

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-cit-landing.report.xlsx
+++ b/tools/importer/reports/import-cit-landing.report.xlsx
@@ -40,7 +40,7 @@
     <t>cit.report.json</t>
   </si>
   <si>
-    <t>["hero-banner","cards-feature","form-contact","columns-media","columns-media","columns-compare"]</t>
+    <t>["hero-banner","cards","form-contact","columns","columns","columns"]</t>
   </si>
   <si>
     <t>cit</t>
@@ -52,7 +52,7 @@
     <t>cit-landing</t>
   </si>
   <si>
-    <t>2026-08-11T12:54:50.945Z</t>
+    <t>2026-08-11T13:17:53.293Z</t>
   </si>
   <si>
     <t>Collective Investment Trusts | Broadridge</t>

</xml_diff>

<commit_message>
Phase 4: migrate 7 core CIT sibling pages
- matrix-cits: cards (offerings variant) with 23 fund tiles + subadvisors
- cit-services, banks-and-trusts, tpas-and-record-keepers, about-us: hero + default-content lists + columns CTA + form
- broker-dealer-platform: hero + cards (feature) 3-tile + columns CTA + form
- financial-advisers: hero + columns (base, 2-col solutions list) + form
- Extend cards parser (offerings branch), columns parser (compare disambiguation + base multi-col), cleanup transformer (list/heading normalization)
- Add cards.offerings CSS variant; per-page templates + import scripts
- David's Model: bulleted lists kept as default content, not blocks

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-cit-landing.report.xlsx
+++ b/tools/importer/reports/import-cit-landing.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="58">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,6 +37,75 @@
     <t>url</t>
   </si>
   <si>
+    <t>about-us.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","columns","form-contact"]</t>
+  </si>
+  <si>
+    <t>about-us</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>2026-08-11T15:36:02.082Z</t>
+  </si>
+  <si>
+    <t>Matrix Trust Company | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/about-us</t>
+  </si>
+  <si>
+    <t>banks-and-trusts.report.json</t>
+  </si>
+  <si>
+    <t>banks-and-trusts</t>
+  </si>
+  <si>
+    <t>2026-08-11T15:24:05.647Z</t>
+  </si>
+  <si>
+    <t>Matrix Banks and Trusts | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/banks-and-trusts</t>
+  </si>
+  <si>
+    <t>broker-dealer-platform.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","cards","columns","form-contact"]</t>
+  </si>
+  <si>
+    <t>broker-dealer-platform</t>
+  </si>
+  <si>
+    <t>2026-08-11T15:35:51.500Z</t>
+  </si>
+  <si>
+    <t>Broker-Dealer Platform | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/broker-dealer-platform</t>
+  </si>
+  <si>
+    <t>cit-services.report.json</t>
+  </si>
+  <si>
+    <t>cit-services</t>
+  </si>
+  <si>
+    <t>2026-08-11T14:50:33.904Z</t>
+  </si>
+  <si>
+    <t>Collective Investment Trust Services | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/cit-services</t>
+  </si>
+  <si>
     <t>cit.report.json</t>
   </si>
   <si>
@@ -46,19 +115,76 @@
     <t>cit</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>cit-landing</t>
   </si>
   <si>
-    <t>2026-08-11T13:17:53.293Z</t>
+    <t>2026-08-11T15:45:17.585Z</t>
   </si>
   <si>
     <t>Collective Investment Trusts | Broadridge</t>
   </si>
   <si>
     <t>https://www.broadridge.com/cit/</t>
+  </si>
+  <si>
+    <t>financial-advisers.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","columns","columns","form-contact"]</t>
+  </si>
+  <si>
+    <t>financial-advisers</t>
+  </si>
+  <si>
+    <t>2026-08-11T15:43:24.842Z</t>
+  </si>
+  <si>
+    <t>Financial Advisers | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/financial-advisers</t>
+  </si>
+  <si>
+    <t>matrix-cits.report.json</t>
+  </si>
+  <si>
+    <t>matrix-cits</t>
+  </si>
+  <si>
+    <t>cit-offerings</t>
+  </si>
+  <si>
+    <t>2026-08-11T15:14:08.996Z</t>
+  </si>
+  <si>
+    <t>Matrix Trust Company Collective Investment Trusts | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/matrix-cits</t>
+  </si>
+  <si>
+    <t>tpas-and-record-keepers.report.json</t>
+  </si>
+  <si>
+    <t>tpas-and-record-keepers</t>
+  </si>
+  <si>
+    <t>2026-08-11T15:34:16.431Z</t>
+  </si>
+  <si>
+    <t>TPAs and Recordkeepers | Broadridge</t>
+  </si>
+  <si>
+    <t>https://www.broadridge.com/cit/tpas-and-record-keepers</t>
+  </si>
+  <si>
+    <t>cit/matrix-cits.report.json</t>
+  </si>
+  <si>
+    <t>cit/matrix-cits</t>
+  </si>
+  <si>
+    <t>2026-08-11T14:30:13.239Z</t>
   </si>
 </sst>
 </file>
@@ -447,16 +573,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="1" max="1" width="37" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="5" max="5" width="25" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="43" customWidth="1"/>
-    <col min="8" max="8" width="33" customWidth="1"/>
+    <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -499,16 +624,224 @@
         <v>11</v>
       </c>
       <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>13</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>14</v>
       </c>
-      <c r="H2" t="s">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>46</v>
+      </c>
+      <c r="F8" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" t="s">
+        <v>48</v>
+      </c>
+      <c r="H8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>51</v>
+      </c>
+      <c r="F9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>46</v>
+      </c>
+      <c r="F10" t="s">
+        <v>57</v>
+      </c>
+      <c r="G10" t="s">
+        <v>48</v>
+      </c>
+      <c r="H10" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix TALK TO US anchor: form-contact block creates #talk-to-us target
- form-contact.js: set id=talk-to-us on the block's section so the nav/tools/
  closing-CTA 'TALK TO US' links (all href=#talk-to-us) scroll to the form
- form-contact.css: scroll-margin-top so the fixed header doesn't cover the
  form on jump
- Content hrefs were already correct (#talk-to-us); the anchor target element
  was missing — this is a code-only fix, no content change needed

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-cit-landing.report.xlsx
+++ b/tools/importer/reports/import-cit-landing.report.xlsx
@@ -55,7 +55,7 @@
     <t>fund-detail</t>
   </si>
   <si>
-    <t>2026-08-12T05:36:56.477Z</t>
+    <t>2026-08-12T05:43:14.235Z</t>
   </si>
   <si>
     <t>3EDGE Asset Management | Broadridge</t>
@@ -73,7 +73,7 @@
     <t>about-us</t>
   </si>
   <si>
-    <t>2026-08-12T05:32:43.386Z</t>
+    <t>2026-08-12T05:42:42.666Z</t>
   </si>
   <si>
     <t>Matrix Trust Company | Broadridge</t>
@@ -88,7 +88,7 @@
     <t>banks-and-trusts</t>
   </si>
   <si>
-    <t>2026-08-12T05:32:18.325Z</t>
+    <t>2026-08-12T05:42:17.067Z</t>
   </si>
   <si>
     <t>Matrix Banks and Trusts | Broadridge</t>
@@ -106,7 +106,7 @@
     <t>broker-dealer-platform</t>
   </si>
   <si>
-    <t>2026-08-12T05:32:10.610Z</t>
+    <t>2026-08-12T05:42:08.883Z</t>
   </si>
   <si>
     <t>Broker-Dealer Platform | Broadridge</t>
@@ -121,7 +121,7 @@
     <t>cit-services</t>
   </si>
   <si>
-    <t>2026-08-12T05:32:02.222Z</t>
+    <t>2026-08-12T05:41:58.902Z</t>
   </si>
   <si>
     <t>Collective Investment Trust Services | Broadridge</t>
@@ -142,7 +142,7 @@
     <t>cit-landing</t>
   </si>
   <si>
-    <t>2026-08-12T05:41:39.515Z</t>
+    <t>2026-08-12T06:20:35.633Z</t>
   </si>
   <si>
     <t>Collective Investment Trusts | Broadridge</t>
@@ -157,7 +157,7 @@
     <t>commerce-core-bond-cit</t>
   </si>
   <si>
-    <t>2026-08-12T05:35:54.034Z</t>
+    <t>2026-08-12T05:42:10.334Z</t>
   </si>
   <si>
     <t>Commerce Core Bond CIT | Broadridge</t>
@@ -172,7 +172,7 @@
     <t>donaldson-preservation-fund</t>
   </si>
   <si>
-    <t>2026-08-12T05:37:09.117Z</t>
+    <t>2026-08-12T05:43:26.116Z</t>
   </si>
   <si>
     <t>Donaldson Preservation Fund | Broadridge</t>
@@ -187,7 +187,7 @@
     <t>donaldson-rising-dividend-fund</t>
   </si>
   <si>
-    <t>2026-08-12T05:37:02.484Z</t>
+    <t>2026-08-12T05:43:20.352Z</t>
   </si>
   <si>
     <t>Donaldson Rising Dividend | Broadridge</t>
@@ -202,7 +202,7 @@
     <t>donaldson-sequoia-fund</t>
   </si>
   <si>
-    <t>2026-08-12T05:36:12.990Z</t>
+    <t>2026-08-12T05:42:30.434Z</t>
   </si>
   <si>
     <t>Donaldson Sequoia Fund | Broadridge</t>
@@ -217,7 +217,7 @@
     <t>equity-armor-cits</t>
   </si>
   <si>
-    <t>2026-08-12T05:35:41.939Z</t>
+    <t>2026-08-12T05:41:55.560Z</t>
   </si>
   <si>
     <t>Equity Armor CITs | Broadridge</t>
@@ -235,7 +235,7 @@
     <t>financial-advisers</t>
   </si>
   <si>
-    <t>2026-08-12T05:32:34.690Z</t>
+    <t>2026-08-12T05:42:34.106Z</t>
   </si>
   <si>
     <t>Financial Advisers | Broadridge</t>
@@ -265,7 +265,7 @@
     <t>goalpath-portfolios</t>
   </si>
   <si>
-    <t>2026-08-12T05:37:21.999Z</t>
+    <t>2026-08-12T05:43:39.509Z</t>
   </si>
   <si>
     <t>GoalPath Portfolios | Broadridge</t>
@@ -280,7 +280,7 @@
     <t>highland-capital-management-core-fixed-fund</t>
   </si>
   <si>
-    <t>2026-08-12T05:36:44.738Z</t>
+    <t>2026-08-12T05:43:01.938Z</t>
   </si>
   <si>
     <t>Highland Capital Management: SMID Cap Core Alpha Fund | Broadridge</t>
@@ -295,7 +295,7 @@
     <t>highland-capital-management-smid-cap-core-alpha-fund</t>
   </si>
   <si>
-    <t>2026-08-12T05:36:37.163Z</t>
+    <t>2026-08-12T05:42:55.989Z</t>
   </si>
   <si>
     <t>https://www.broadridge.com/cit/highland-capital-management-smid-cap-core-alpha-fund</t>
@@ -307,7 +307,7 @@
     <t>managed-retirement-funds</t>
   </si>
   <si>
-    <t>2026-08-12T05:37:28.436Z</t>
+    <t>2026-08-12T05:43:47.597Z</t>
   </si>
   <si>
     <t>Managed Retirement Funds | Broadridge</t>
@@ -325,7 +325,7 @@
     <t>cit-offerings</t>
   </si>
   <si>
-    <t>2026-08-12T05:31:54.558Z</t>
+    <t>2026-08-12T05:41:48.694Z</t>
   </si>
   <si>
     <t>Matrix Trust Company Collective Investment Trusts | Broadridge</t>
@@ -340,7 +340,7 @@
     <t>matrix-trust-multi-manager-stable-value-fund</t>
   </si>
   <si>
-    <t>2026-08-12T05:37:15.545Z</t>
+    <t>2026-08-12T05:43:32.875Z</t>
   </si>
   <si>
     <t>Matrix Trust Multi Manager Stable Value Fund | Broadridge</t>
@@ -355,7 +355,7 @@
     <t>mtc-northern-trust</t>
   </si>
   <si>
-    <t>2026-08-12T05:36:19.291Z</t>
+    <t>2026-08-12T05:42:37.637Z</t>
   </si>
   <si>
     <t>MTC Northern Trust Index | Broadridge</t>
@@ -397,7 +397,7 @@
     <t>pacific-life-income-horizon-cits</t>
   </si>
   <si>
-    <t>2026-08-12T05:35:34.836Z</t>
+    <t>2026-08-12T05:41:47.781Z</t>
   </si>
   <si>
     <t>Pacific Life Income Horizon CITs | Broadridge</t>
@@ -412,7 +412,7 @@
     <t>pacific-ridge-small-cap-value</t>
   </si>
   <si>
-    <t>2026-08-12T05:35:48.679Z</t>
+    <t>2026-08-12T05:42:03.335Z</t>
   </si>
   <si>
     <t>Pacific Ridge Small Cap Value | Broadridge</t>
@@ -427,7 +427,7 @@
     <t>retirement-advocate-funds</t>
   </si>
   <si>
-    <t>2026-08-12T05:37:34.403Z</t>
+    <t>2026-08-12T05:43:55.022Z</t>
   </si>
   <si>
     <t>Retirement Advocate Funds | Broadridge</t>
@@ -445,7 +445,7 @@
     <t>starpath-funds</t>
   </si>
   <si>
-    <t>2026-08-12T05:37:40.474Z</t>
+    <t>2026-08-12T05:44:01.972Z</t>
   </si>
   <si>
     <t>StarPath Funds | Broadridge</t>
@@ -460,7 +460,7 @@
     <t>strategic-roadmap-portfolios</t>
   </si>
   <si>
-    <t>2026-08-12T05:37:48.206Z</t>
+    <t>2026-08-12T05:44:08.455Z</t>
   </si>
   <si>
     <t>Strategic Roadmap Portfolios | Broadridge</t>
@@ -481,7 +481,7 @@
     <t>legal</t>
   </si>
   <si>
-    <t>2026-08-12T05:32:50.455Z</t>
+    <t>2026-08-12T05:42:51.292Z</t>
   </si>
   <si>
     <t>Matrix Terms of Service</t>
@@ -496,7 +496,7 @@
     <t>tpas-and-record-keepers</t>
   </si>
   <si>
-    <t>2026-08-12T05:32:26.824Z</t>
+    <t>2026-08-12T05:42:24.952Z</t>
   </si>
   <si>
     <t>TPAs and Recordkeepers | Broadridge</t>
@@ -511,7 +511,7 @@
     <t>twelve-points-retirement-advisors-100-percent-equity-fund</t>
   </si>
   <si>
-    <t>2026-08-12T05:36:24.138Z</t>
+    <t>2026-08-12T05:42:43.074Z</t>
   </si>
   <si>
     <t>Twelve Points Retirement Advisors 100% Equity Fund | Broadridge</t>
@@ -526,7 +526,7 @@
     <t>twelve-points-target-risk-portfolios</t>
   </si>
   <si>
-    <t>2026-08-12T05:36:30.775Z</t>
+    <t>2026-08-12T05:42:50.735Z</t>
   </si>
   <si>
     <t>Twelve Points Target Risk Portfolios | Broadridge</t>
@@ -541,7 +541,7 @@
     <t>wealthplan-partners-dividend-aristocrats-portfolio-fund</t>
   </si>
   <si>
-    <t>2026-08-12T05:36:50.243Z</t>
+    <t>2026-08-12T05:43:07.499Z</t>
   </si>
   <si>
     <t>WealthPlan Partners Dividend Aristocrats Portfolio Fund | Broadridge</t>
@@ -556,7 +556,7 @@
     <t>xponance-inc-small-cap-core-equity-smid-cap-core-equity-funds</t>
   </si>
   <si>
-    <t>2026-08-12T05:36:06.155Z</t>
+    <t>2026-08-12T05:42:23.559Z</t>
   </si>
   <si>
     <t>Xponance Inc. Small Cap Core Equity/SMID Cap Core Equity Funds | Broadridge</t>
@@ -571,7 +571,7 @@
     <t>xponance-inc-yield-advantage-opportunistic-core-bond-fund</t>
   </si>
   <si>
-    <t>2026-08-12T05:36:00.437Z</t>
+    <t>2026-08-12T05:42:16.932Z</t>
   </si>
   <si>
     <t>Xponance Inc. Yield Advantage Opportunistic Core Bond Fund | Broadridge</t>

</xml_diff>